<commit_message>
Expand CDR template and name school workbooks
</commit_message>
<xml_diff>
--- a/assets/cdr_template.xlsx
+++ b/assets/cdr_template.xlsx
@@ -17,6 +17,10 @@
     <sheet name="UACS" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabacungan ES-Q1'!$A$1:$L$95</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cabacungan ES-Q1'!$14:$18</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -1364,7 +1368,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:AU88"/>
+  <dimension ref="A2:AU100"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="22.140625" customWidth="1"/>
@@ -4606,33 +4610,18 @@
       <c r="AT56" s="2"/>
       <c r="AU56" s="2"/>
     </row>
-    <row r="57" spans="1:47" ht="15">
-      <c r="A57" s="66"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="68" t="s">
-        <v>98</v>
-      </c>
-      <c r="D57" s="69"/>
-      <c r="E57" s="69"/>
-      <c r="F57" s="69"/>
-      <c r="G57" s="70">
-        <f t="shared" ref="G57:I57" si="1">SUM(G20:G56)</f>
-        <v>60594.17</v>
-      </c>
-      <c r="H57" s="70">
-        <f t="shared" si="1"/>
-        <v>41000</v>
-      </c>
-      <c r="I57" s="70">
-        <f t="shared" si="1"/>
-        <v>21000</v>
-      </c>
-      <c r="J57" s="71"/>
-      <c r="K57" s="70"/>
-      <c r="L57" s="70">
-        <f>SUM(L21:L56)</f>
-        <v>131155.83000000002</v>
-      </c>
+    <row r="57" spans="1:47" ht="25.5">
+      <c r="A57" s="51"/>
+      <c r="B57" s="65"/>
+      <c r="C57" s="53"/>
+      <c r="D57" s="59"/>
+      <c r="F57" s="26"/>
+      <c r="G57" s="32"/>
+      <c r="H57" s="42"/>
+      <c r="I57" s="42"/>
+      <c r="J57" s="28"/>
+      <c r="K57" s="29"/>
+      <c r="L57" s="32"/>
       <c r="M57" s="2"/>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -4669,19 +4658,18 @@
       <c r="AT57" s="2"/>
       <c r="AU57" s="2"/>
     </row>
-    <row r="58" spans="1:47" ht="12.75">
-      <c r="A58" s="66"/>
-      <c r="B58" s="67"/>
-      <c r="C58" s="67"/>
-      <c r="D58" s="72"/>
-      <c r="E58" s="72"/>
-      <c r="F58" s="72"/>
-      <c r="G58" s="72"/>
-      <c r="H58" s="72"/>
-      <c r="I58" s="72"/>
-      <c r="J58" s="72"/>
-      <c r="K58" s="72"/>
-      <c r="L58" s="73"/>
+    <row r="58" spans="1:47" ht="25.5">
+      <c r="A58" s="51"/>
+      <c r="B58" s="65"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="59"/>
+      <c r="F58" s="26"/>
+      <c r="G58" s="32"/>
+      <c r="H58" s="42"/>
+      <c r="I58" s="42"/>
+      <c r="J58" s="28"/>
+      <c r="K58" s="29"/>
+      <c r="L58" s="32"/>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -4718,21 +4706,18 @@
       <c r="AT58" s="2"/>
       <c r="AU58" s="2"/>
     </row>
-    <row r="59" spans="1:47" ht="12.75">
-      <c r="A59" s="66"/>
-      <c r="B59" s="67"/>
-      <c r="C59" s="67"/>
-      <c r="D59" s="72"/>
-      <c r="E59" s="72"/>
-      <c r="F59" s="72"/>
-      <c r="G59" s="72"/>
-      <c r="H59" s="72"/>
-      <c r="I59" s="72"/>
-      <c r="J59" s="74" t="s">
-        <v>99</v>
-      </c>
-      <c r="K59" s="75"/>
-      <c r="L59" s="76"/>
+    <row r="59" spans="1:47" ht="25.5">
+      <c r="A59" s="51"/>
+      <c r="B59" s="65"/>
+      <c r="C59" s="53"/>
+      <c r="D59" s="59"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="32"/>
+      <c r="H59" s="42"/>
+      <c r="I59" s="42"/>
+      <c r="J59" s="28"/>
+      <c r="K59" s="29"/>
+      <c r="L59" s="32"/>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -4769,25 +4754,18 @@
       <c r="AT59" s="2"/>
       <c r="AU59" s="2"/>
     </row>
-    <row r="60" spans="1:47" ht="12.75">
-      <c r="A60" s="66"/>
-      <c r="B60" s="67"/>
-      <c r="C60" s="67"/>
-      <c r="D60" s="72"/>
-      <c r="E60" s="72"/>
-      <c r="F60" s="72"/>
-      <c r="G60" s="72"/>
-      <c r="H60" s="72"/>
-      <c r="I60" s="72"/>
-      <c r="J60" s="77" t="s">
-        <v>26</v>
-      </c>
-      <c r="K60" s="78" t="s">
-        <v>27</v>
-      </c>
-      <c r="L60" s="77" t="s">
-        <v>18</v>
-      </c>
+    <row r="60" spans="1:47" ht="25.5">
+      <c r="A60" s="51"/>
+      <c r="B60" s="65"/>
+      <c r="C60" s="53"/>
+      <c r="D60" s="59"/>
+      <c r="F60" s="26"/>
+      <c r="G60" s="32"/>
+      <c r="H60" s="42"/>
+      <c r="I60" s="42"/>
+      <c r="J60" s="28"/>
+      <c r="K60" s="29"/>
+      <c r="L60" s="32"/>
       <c r="M60" s="2"/>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -4824,26 +4802,18 @@
       <c r="AT60" s="2"/>
       <c r="AU60" s="2"/>
     </row>
-    <row r="61" spans="1:47" ht="12.75">
-      <c r="A61" s="66"/>
-      <c r="B61" s="67"/>
-      <c r="C61" s="67"/>
-      <c r="D61" s="72"/>
-      <c r="E61" s="72"/>
-      <c r="F61" s="72"/>
-      <c r="G61" s="72"/>
-      <c r="H61" s="72"/>
-      <c r="I61" s="72"/>
-      <c r="J61" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="K61" s="64">
-        <v>5020503000</v>
-      </c>
-      <c r="L61" s="32">
-        <f>SUMIF(J19:J58, "Internet Subcription Expenses", L19:L58)</f>
-        <v>11501</v>
-      </c>
+    <row r="61" spans="1:47" ht="25.5">
+      <c r="A61" s="51"/>
+      <c r="B61" s="65"/>
+      <c r="C61" s="53"/>
+      <c r="D61" s="59"/>
+      <c r="F61" s="26"/>
+      <c r="G61" s="32"/>
+      <c r="H61" s="42"/>
+      <c r="I61" s="42"/>
+      <c r="J61" s="28"/>
+      <c r="K61" s="29"/>
+      <c r="L61" s="32"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
@@ -4880,26 +4850,18 @@
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
     </row>
-    <row r="62" spans="1:47" ht="12.75">
-      <c r="A62" s="66"/>
-      <c r="B62" s="67"/>
-      <c r="C62" s="67"/>
-      <c r="D62" s="72"/>
-      <c r="E62" s="72"/>
-      <c r="F62" s="72"/>
-      <c r="G62" s="72"/>
-      <c r="H62" s="72"/>
-      <c r="I62" s="72"/>
-      <c r="J62" s="79" t="s">
-        <v>41</v>
-      </c>
-      <c r="K62" s="80">
-        <v>5020402000</v>
-      </c>
-      <c r="L62" s="32">
-        <f>SUMIF(J19:J58, "Electricity Expenses", L19:L58)</f>
-        <v>32161.829999999998</v>
-      </c>
+    <row r="62" spans="1:47" ht="25.5">
+      <c r="A62" s="51"/>
+      <c r="B62" s="65"/>
+      <c r="C62" s="53"/>
+      <c r="D62" s="59"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="32"/>
+      <c r="H62" s="42"/>
+      <c r="I62" s="42"/>
+      <c r="J62" s="28"/>
+      <c r="K62" s="29"/>
+      <c r="L62" s="32"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -4936,26 +4898,18 @@
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
     </row>
-    <row r="63" spans="1:47" ht="12.75">
-      <c r="A63" s="66"/>
-      <c r="B63" s="67"/>
-      <c r="C63" s="67"/>
-      <c r="D63" s="72"/>
-      <c r="E63" s="72"/>
-      <c r="F63" s="72"/>
-      <c r="G63" s="72"/>
-      <c r="H63" s="72"/>
-      <c r="I63" s="72"/>
-      <c r="J63" s="81" t="s">
-        <v>44</v>
-      </c>
-      <c r="K63" s="64">
-        <v>5020101000</v>
-      </c>
-      <c r="L63" s="32">
-        <f>SUMIF(J9:J58, "Travelling Expenses-Local", L9:L58)</f>
-        <v>3760</v>
-      </c>
+    <row r="63" spans="1:47" ht="25.5">
+      <c r="A63" s="51"/>
+      <c r="B63" s="65"/>
+      <c r="C63" s="53"/>
+      <c r="D63" s="59"/>
+      <c r="F63" s="26"/>
+      <c r="G63" s="32"/>
+      <c r="H63" s="42"/>
+      <c r="I63" s="42"/>
+      <c r="J63" s="28"/>
+      <c r="K63" s="29"/>
+      <c r="L63" s="32"/>
       <c r="M63" s="2"/>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -4992,26 +4946,18 @@
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
     </row>
-    <row r="64" spans="1:47" ht="12.75">
-      <c r="A64" s="66"/>
-      <c r="B64" s="67"/>
-      <c r="C64" s="67"/>
-      <c r="D64" s="72"/>
-      <c r="E64" s="72"/>
-      <c r="F64" s="72"/>
-      <c r="G64" s="72"/>
-      <c r="H64" s="72"/>
-      <c r="I64" s="72"/>
-      <c r="J64" s="81" t="s">
-        <v>62</v>
-      </c>
-      <c r="K64" s="82">
-        <v>5020502001</v>
-      </c>
-      <c r="L64" s="32">
-        <f>SUMIF(J1:J58, "Accountable Forms", L1:L58)</f>
-        <v>1200</v>
-      </c>
+    <row r="64" spans="1:47" ht="25.5">
+      <c r="A64" s="51"/>
+      <c r="B64" s="65"/>
+      <c r="C64" s="53"/>
+      <c r="D64" s="59"/>
+      <c r="F64" s="26"/>
+      <c r="G64" s="32"/>
+      <c r="H64" s="42"/>
+      <c r="I64" s="42"/>
+      <c r="J64" s="28"/>
+      <c r="K64" s="29"/>
+      <c r="L64" s="32"/>
       <c r="M64" s="2"/>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -5049,25 +4995,17 @@
       <c r="AU64" s="2"/>
     </row>
     <row r="65" spans="1:47" ht="25.5">
-      <c r="A65" s="66"/>
-      <c r="B65" s="67"/>
-      <c r="C65" s="67"/>
-      <c r="D65" s="72"/>
-      <c r="E65" s="72"/>
-      <c r="F65" s="72"/>
-      <c r="G65" s="72"/>
-      <c r="H65" s="72"/>
-      <c r="I65" s="72"/>
-      <c r="J65" s="81" t="s">
-        <v>63</v>
-      </c>
-      <c r="K65" s="64">
-        <v>5029902000</v>
-      </c>
-      <c r="L65" s="32">
-        <f>SUMIF(J1:J58, "Printing and Publication Expenses", L1:L58)</f>
-        <v>3020</v>
-      </c>
+      <c r="A65" s="51"/>
+      <c r="B65" s="65"/>
+      <c r="C65" s="53"/>
+      <c r="D65" s="59"/>
+      <c r="F65" s="26"/>
+      <c r="G65" s="32"/>
+      <c r="H65" s="42"/>
+      <c r="I65" s="42"/>
+      <c r="J65" s="28"/>
+      <c r="K65" s="29"/>
+      <c r="L65" s="32"/>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -5105,25 +5043,17 @@
       <c r="AU65" s="2"/>
     </row>
     <row r="66" spans="1:47" ht="25.5">
-      <c r="A66" s="66"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67"/>
-      <c r="D66" s="72"/>
-      <c r="E66" s="72"/>
-      <c r="F66" s="72"/>
-      <c r="G66" s="72"/>
-      <c r="H66" s="72"/>
-      <c r="I66" s="72"/>
-      <c r="J66" s="48" t="s">
-        <v>50</v>
-      </c>
-      <c r="K66" s="64">
-        <v>5020399000</v>
-      </c>
-      <c r="L66" s="32">
-        <f>SUMIF(J1:J58, "Other Supplies and Materials Expenses", L1:L58)</f>
-        <v>72498</v>
-      </c>
+      <c r="A66" s="51"/>
+      <c r="B66" s="65"/>
+      <c r="C66" s="53"/>
+      <c r="D66" s="59"/>
+      <c r="F66" s="26"/>
+      <c r="G66" s="32"/>
+      <c r="H66" s="42"/>
+      <c r="I66" s="42"/>
+      <c r="J66" s="28"/>
+      <c r="K66" s="29"/>
+      <c r="L66" s="32"/>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -5161,25 +5091,17 @@
       <c r="AU66" s="2"/>
     </row>
     <row r="67" spans="1:47" ht="25.5">
-      <c r="A67" s="66"/>
-      <c r="B67" s="67"/>
-      <c r="C67" s="67"/>
-      <c r="D67" s="72"/>
-      <c r="E67" s="72"/>
-      <c r="F67" s="72"/>
-      <c r="G67" s="72"/>
-      <c r="H67" s="72"/>
-      <c r="I67" s="72"/>
-      <c r="J67" s="48" t="s">
-        <v>73</v>
-      </c>
-      <c r="K67" s="64">
-        <v>5021305002</v>
-      </c>
-      <c r="L67" s="32">
-        <f>SUMIF(J2:J59, "Repairs and Maintenance-Office Equipment", L2:L59)</f>
-        <v>3850</v>
-      </c>
+      <c r="A67" s="51"/>
+      <c r="B67" s="65"/>
+      <c r="C67" s="53"/>
+      <c r="D67" s="59"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="32"/>
+      <c r="H67" s="42"/>
+      <c r="I67" s="42"/>
+      <c r="J67" s="28"/>
+      <c r="K67" s="29"/>
+      <c r="L67" s="32"/>
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
@@ -5216,26 +5138,18 @@
       <c r="AT67" s="2"/>
       <c r="AU67" s="2"/>
     </row>
-    <row r="68" spans="1:47" ht="12.75">
-      <c r="A68" s="66"/>
-      <c r="B68" s="67"/>
-      <c r="C68" s="67"/>
-      <c r="D68" s="72"/>
-      <c r="E68" s="72"/>
-      <c r="F68" s="72"/>
-      <c r="G68" s="72"/>
-      <c r="H68" s="72"/>
-      <c r="I68" s="72"/>
-      <c r="J68" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="K68" s="64">
-        <v>5020201000</v>
-      </c>
-      <c r="L68" s="32">
-        <f>SUMIF(J3:J60, "Training Expenses", L3:L60)</f>
-        <v>2990</v>
-      </c>
+    <row r="68" spans="1:47" ht="25.5">
+      <c r="A68" s="51"/>
+      <c r="B68" s="65"/>
+      <c r="C68" s="53"/>
+      <c r="D68" s="59"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="32"/>
+      <c r="H68" s="42"/>
+      <c r="I68" s="42"/>
+      <c r="J68" s="28"/>
+      <c r="K68" s="29"/>
+      <c r="L68" s="32"/>
       <c r="M68" s="2"/>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -5272,24 +5186,32 @@
       <c r="AT68" s="2"/>
       <c r="AU68" s="2"/>
     </row>
-    <row r="69" spans="1:47" ht="12.75">
+    <row r="69" spans="1:47" ht="15">
       <c r="A69" s="66"/>
       <c r="B69" s="67"/>
-      <c r="C69" s="67"/>
-      <c r="D69" s="72"/>
-      <c r="E69" s="72"/>
-      <c r="F69" s="72"/>
-      <c r="G69" s="72"/>
-      <c r="H69" s="72"/>
-      <c r="I69" s="72"/>
-      <c r="J69" s="45" t="s">
-        <v>95</v>
-      </c>
-      <c r="K69" s="64">
-        <v>5020501000</v>
-      </c>
-      <c r="L69" s="83">
-        <v>175</v>
+      <c r="C69" s="68" t="s">
+        <v>98</v>
+      </c>
+      <c r="D69" s="69"/>
+      <c r="E69" s="69"/>
+      <c r="F69" s="69"/>
+      <c r="G69" s="70">
+        <f t="shared" ref="G57:I57" si="1">SUM(G20:G68)</f>
+        <v>60594.17</v>
+      </c>
+      <c r="H69" s="70">
+        <f t="shared" si="1"/>
+        <v>41000</v>
+      </c>
+      <c r="I81" s="70">
+        <f t="shared" si="1"/>
+        <v>21000</v>
+      </c>
+      <c r="J81" s="71"/>
+      <c r="K81" s="70"/>
+      <c r="L81" s="70">
+        <f>SUM(L19:L68)</f>
+        <v>131155.83000000002</v>
       </c>
       <c r="M69" s="2"/>
       <c r="N69" s="2"/>
@@ -5337,9 +5259,9 @@
       <c r="G70" s="72"/>
       <c r="H70" s="72"/>
       <c r="I70" s="72"/>
-      <c r="J70" s="137"/>
-      <c r="K70" s="138"/>
-      <c r="L70" s="139"/>
+      <c r="J70" s="72"/>
+      <c r="K70" s="72"/>
+      <c r="L70" s="73"/>
       <c r="M70" s="2"/>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -5386,9 +5308,11 @@
       <c r="G71" s="72"/>
       <c r="H71" s="72"/>
       <c r="I71" s="72"/>
-      <c r="J71" s="137"/>
-      <c r="K71" s="138"/>
-      <c r="L71" s="139"/>
+      <c r="J71" s="74" t="s">
+        <v>99</v>
+      </c>
+      <c r="K71" s="75"/>
+      <c r="L71" s="76"/>
       <c r="M71" s="2"/>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -5435,9 +5359,15 @@
       <c r="G72" s="72"/>
       <c r="H72" s="72"/>
       <c r="I72" s="72"/>
-      <c r="J72" s="137"/>
-      <c r="K72" s="138"/>
-      <c r="L72" s="139"/>
+      <c r="J72" s="77" t="s">
+        <v>26</v>
+      </c>
+      <c r="K72" s="78" t="s">
+        <v>27</v>
+      </c>
+      <c r="L72" s="77" t="s">
+        <v>18</v>
+      </c>
       <c r="M72" s="2"/>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -5484,9 +5414,16 @@
       <c r="G73" s="72"/>
       <c r="H73" s="72"/>
       <c r="I73" s="72"/>
-      <c r="J73" s="137"/>
-      <c r="K73" s="138"/>
-      <c r="L73" s="139"/>
+      <c r="J73" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="K73" s="64">
+        <v>5020503000</v>
+      </c>
+      <c r="L73" s="32">
+        <f>SUMIF(J19:J68, "Internet Subcription Expenses", L19:L68)</f>
+        <v>11501</v>
+      </c>
       <c r="M73" s="2"/>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
@@ -5533,9 +5470,16 @@
       <c r="G74" s="72"/>
       <c r="H74" s="72"/>
       <c r="I74" s="72"/>
-      <c r="J74" s="137"/>
-      <c r="K74" s="138"/>
-      <c r="L74" s="139"/>
+      <c r="J74" s="79" t="s">
+        <v>41</v>
+      </c>
+      <c r="K74" s="80">
+        <v>5020402000</v>
+      </c>
+      <c r="L74" s="32">
+        <f>SUMIF(J19:J68, "Electricity Expenses", L19:L68)</f>
+        <v>32161.829999999998</v>
+      </c>
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -5576,19 +5520,21 @@
       <c r="A75" s="66"/>
       <c r="B75" s="67"/>
       <c r="C75" s="67"/>
-      <c r="D75" s="84"/>
+      <c r="D75" s="72"/>
       <c r="E75" s="72"/>
       <c r="F75" s="72"/>
       <c r="G75" s="72"/>
       <c r="H75" s="72"/>
       <c r="I75" s="72"/>
-      <c r="J75" s="85" t="s">
-        <v>100</v>
-      </c>
-      <c r="K75" s="86"/>
-      <c r="L75" s="87">
-        <f>SUM(L61:L69)</f>
-        <v>131155.83000000002</v>
+      <c r="J75" s="81" t="s">
+        <v>44</v>
+      </c>
+      <c r="K75" s="64">
+        <v>5020101000</v>
+      </c>
+      <c r="L75" s="32">
+        <f>SUMIF(J19:J68, "Travelling Expenses-Local", L19:L68)</f>
+        <v>3760</v>
       </c>
       <c r="M75" s="2"/>
       <c r="N75" s="2"/>
@@ -5626,21 +5572,26 @@
       <c r="AT75" s="2"/>
       <c r="AU75" s="2"/>
     </row>
-    <row r="76" spans="1:47" ht="14.25">
-      <c r="A76" s="88"/>
-      <c r="B76" s="89"/>
-      <c r="C76" s="89"/>
-      <c r="D76" s="89"/>
-      <c r="E76" s="89"/>
-      <c r="F76" s="90"/>
-      <c r="G76" s="135" t="s">
-        <v>101</v>
-      </c>
-      <c r="H76" s="116"/>
-      <c r="I76" s="116"/>
-      <c r="J76" s="116"/>
-      <c r="K76" s="116"/>
-      <c r="L76" s="117"/>
+    <row r="76" spans="1:47" ht="12.75">
+      <c r="A76" s="66"/>
+      <c r="B76" s="67"/>
+      <c r="C76" s="67"/>
+      <c r="D76" s="72"/>
+      <c r="E76" s="72"/>
+      <c r="F76" s="72"/>
+      <c r="G76" s="72"/>
+      <c r="H76" s="72"/>
+      <c r="I76" s="72"/>
+      <c r="J76" s="81" t="s">
+        <v>62</v>
+      </c>
+      <c r="K76" s="82">
+        <v>5020502001</v>
+      </c>
+      <c r="L76" s="32">
+        <f>SUMIF(J19:J68, "Accountable Forms", L19:L68)</f>
+        <v>1200</v>
+      </c>
       <c r="M76" s="2"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -5677,19 +5628,26 @@
       <c r="AT76" s="2"/>
       <c r="AU76" s="2"/>
     </row>
-    <row r="77" spans="1:47" ht="14.25">
-      <c r="A77" s="91"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="92"/>
-      <c r="G77" s="9"/>
-      <c r="H77" s="9"/>
-      <c r="I77" s="9"/>
-      <c r="J77" s="9"/>
-      <c r="K77" s="9"/>
-      <c r="L77" s="93"/>
+    <row r="77" spans="1:47" ht="25.5">
+      <c r="A77" s="66"/>
+      <c r="B77" s="67"/>
+      <c r="C77" s="67"/>
+      <c r="D77" s="72"/>
+      <c r="E77" s="72"/>
+      <c r="F77" s="72"/>
+      <c r="G77" s="72"/>
+      <c r="H77" s="72"/>
+      <c r="I77" s="72"/>
+      <c r="J77" s="81" t="s">
+        <v>63</v>
+      </c>
+      <c r="K77" s="64">
+        <v>5029902000</v>
+      </c>
+      <c r="L77" s="32">
+        <f>SUMIF(J19:J68, "Printing and Publication Expenses", L19:L68)</f>
+        <v>3020</v>
+      </c>
       <c r="M77" s="2"/>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
@@ -5726,23 +5684,26 @@
       <c r="AT77" s="2"/>
       <c r="AU77" s="2"/>
     </row>
-    <row r="78" spans="1:47" ht="14.25">
-      <c r="A78" s="94"/>
-      <c r="B78" s="127" t="s">
-        <v>102</v>
-      </c>
-      <c r="C78" s="107"/>
-      <c r="D78" s="9"/>
-      <c r="E78" s="9"/>
-      <c r="F78" s="92"/>
-      <c r="G78" s="9"/>
-      <c r="H78" s="136" t="s">
-        <v>103</v>
-      </c>
-      <c r="I78" s="107"/>
-      <c r="J78" s="9"/>
-      <c r="K78" s="9"/>
-      <c r="L78" s="93"/>
+    <row r="78" spans="1:47" ht="25.5">
+      <c r="A78" s="66"/>
+      <c r="B78" s="67"/>
+      <c r="C78" s="67"/>
+      <c r="D78" s="72"/>
+      <c r="E78" s="72"/>
+      <c r="F78" s="72"/>
+      <c r="G78" s="72"/>
+      <c r="H78" s="72"/>
+      <c r="I78" s="72"/>
+      <c r="J78" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K78" s="64">
+        <v>5020399000</v>
+      </c>
+      <c r="L78" s="32">
+        <f>SUMIF(J19:J68, "Other Supplies and Materials Expenses", L19:L68)</f>
+        <v>72498</v>
+      </c>
       <c r="M78" s="2"/>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -5779,19 +5740,26 @@
       <c r="AT78" s="2"/>
       <c r="AU78" s="2"/>
     </row>
-    <row r="79" spans="1:47" ht="14.25">
-      <c r="A79" s="94"/>
-      <c r="B79" s="95"/>
-      <c r="C79" s="95"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="9"/>
-      <c r="F79" s="92"/>
-      <c r="G79" s="9"/>
-      <c r="H79" s="96"/>
-      <c r="I79" s="96"/>
-      <c r="J79" s="9"/>
-      <c r="K79" s="9"/>
-      <c r="L79" s="93"/>
+    <row r="79" spans="1:47" ht="25.5">
+      <c r="A79" s="66"/>
+      <c r="B79" s="67"/>
+      <c r="C79" s="67"/>
+      <c r="D79" s="72"/>
+      <c r="E79" s="72"/>
+      <c r="F79" s="72"/>
+      <c r="G79" s="72"/>
+      <c r="H79" s="72"/>
+      <c r="I79" s="72"/>
+      <c r="J79" s="48" t="s">
+        <v>73</v>
+      </c>
+      <c r="K79" s="64">
+        <v>5021305002</v>
+      </c>
+      <c r="L79" s="32">
+        <f>SUMIF(J19:J68, "Repairs and Maintenance-Office Equipment", L19:L68)</f>
+        <v>3850</v>
+      </c>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
@@ -5828,23 +5796,26 @@
       <c r="AT79" s="2"/>
       <c r="AU79" s="2"/>
     </row>
-    <row r="80" spans="1:47" ht="15">
-      <c r="A80" s="91"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="97" t="s">
-        <v>104</v>
-      </c>
-      <c r="D80" s="9"/>
-      <c r="E80" s="9"/>
-      <c r="F80" s="92"/>
-      <c r="G80" s="9"/>
-      <c r="H80" s="98"/>
-      <c r="I80" s="132" t="s">
-        <v>105</v>
-      </c>
-      <c r="J80" s="107"/>
-      <c r="K80" s="9"/>
-      <c r="L80" s="93"/>
+    <row r="80" spans="1:47" ht="12.75">
+      <c r="A80" s="66"/>
+      <c r="B80" s="67"/>
+      <c r="C80" s="67"/>
+      <c r="D80" s="72"/>
+      <c r="E80" s="72"/>
+      <c r="F80" s="72"/>
+      <c r="G80" s="72"/>
+      <c r="H80" s="72"/>
+      <c r="I80" s="72"/>
+      <c r="J80" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="K80" s="64">
+        <v>5020201000</v>
+      </c>
+      <c r="L80" s="32">
+        <f>SUMIF(J19:J68, "Training Expenses", L19:L68)</f>
+        <v>2990</v>
+      </c>
       <c r="M80" s="2"/>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -5881,23 +5852,25 @@
       <c r="AT80" s="2"/>
       <c r="AU80" s="2"/>
     </row>
-    <row r="81" spans="1:47" ht="14.25">
-      <c r="A81" s="91"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="99" t="s">
-        <v>106</v>
-      </c>
-      <c r="D81" s="9"/>
-      <c r="E81" s="9"/>
-      <c r="F81" s="92"/>
-      <c r="G81" s="9"/>
-      <c r="H81" s="9"/>
-      <c r="I81" s="133" t="s">
-        <v>107</v>
-      </c>
-      <c r="J81" s="107"/>
-      <c r="K81" s="9"/>
-      <c r="L81" s="93"/>
+    <row r="81" spans="1:47" ht="12.75">
+      <c r="A81" s="66"/>
+      <c r="B81" s="67"/>
+      <c r="C81" s="67"/>
+      <c r="D81" s="72"/>
+      <c r="E81" s="72"/>
+      <c r="F81" s="72"/>
+      <c r="G81" s="72"/>
+      <c r="H81" s="72"/>
+      <c r="I81" s="72"/>
+      <c r="J81" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="K81" s="64">
+        <v>5020501000</v>
+      </c>
+      <c r="L81" s="83">
+        <v>175</v>
+      </c>
       <c r="M81" s="2"/>
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
@@ -5934,19 +5907,19 @@
       <c r="AT81" s="2"/>
       <c r="AU81" s="2"/>
     </row>
-    <row r="82" spans="1:47" ht="14.25">
-      <c r="A82" s="91"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
-      <c r="D82" s="9"/>
-      <c r="E82" s="9"/>
-      <c r="F82" s="92"/>
-      <c r="G82" s="9"/>
-      <c r="H82" s="9"/>
-      <c r="I82" s="9"/>
-      <c r="J82" s="9"/>
-      <c r="K82" s="9"/>
-      <c r="L82" s="93"/>
+    <row r="82" spans="1:47" ht="12.75">
+      <c r="A82" s="66"/>
+      <c r="B82" s="67"/>
+      <c r="C82" s="67"/>
+      <c r="D82" s="72"/>
+      <c r="E82" s="72"/>
+      <c r="F82" s="72"/>
+      <c r="G82" s="72"/>
+      <c r="H82" s="72"/>
+      <c r="I82" s="72"/>
+      <c r="J82" s="137"/>
+      <c r="K82" s="138"/>
+      <c r="L82" s="139"/>
       <c r="M82" s="2"/>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -5983,23 +5956,19 @@
       <c r="AT82" s="2"/>
       <c r="AU82" s="2"/>
     </row>
-    <row r="83" spans="1:47" ht="14.25">
-      <c r="A83" s="88"/>
-      <c r="B83" s="89"/>
-      <c r="C83" s="134" t="s">
-        <v>108</v>
-      </c>
-      <c r="D83" s="113"/>
-      <c r="E83" s="113"/>
-      <c r="F83" s="90"/>
-      <c r="G83" s="89"/>
-      <c r="H83" s="89"/>
-      <c r="I83" s="134" t="s">
-        <v>109</v>
-      </c>
-      <c r="J83" s="113"/>
-      <c r="K83" s="89"/>
-      <c r="L83" s="100"/>
+    <row r="83" spans="1:47" ht="12.75">
+      <c r="A83" s="66"/>
+      <c r="B83" s="67"/>
+      <c r="C83" s="67"/>
+      <c r="D83" s="72"/>
+      <c r="E83" s="72"/>
+      <c r="F83" s="72"/>
+      <c r="G83" s="72"/>
+      <c r="H83" s="72"/>
+      <c r="I83" s="72"/>
+      <c r="J83" s="137"/>
+      <c r="K83" s="138"/>
+      <c r="L83" s="139"/>
       <c r="M83" s="2"/>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -6037,18 +6006,18 @@
       <c r="AU83" s="2"/>
     </row>
     <row r="84" spans="1:47" ht="12.75">
-      <c r="A84" s="1"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
-      <c r="H84" s="2"/>
-      <c r="I84" s="2"/>
-      <c r="J84" s="2"/>
-      <c r="K84" s="2"/>
-      <c r="L84" s="2"/>
+      <c r="A84" s="66"/>
+      <c r="B84" s="67"/>
+      <c r="C84" s="67"/>
+      <c r="D84" s="72"/>
+      <c r="E84" s="72"/>
+      <c r="F84" s="72"/>
+      <c r="G84" s="72"/>
+      <c r="H84" s="72"/>
+      <c r="I84" s="72"/>
+      <c r="J84" s="137"/>
+      <c r="K84" s="138"/>
+      <c r="L84" s="139"/>
       <c r="M84" s="2"/>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -6086,18 +6055,18 @@
       <c r="AU84" s="2"/>
     </row>
     <row r="85" spans="1:47" ht="12.75">
-      <c r="A85" s="1"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
-      <c r="H85" s="2"/>
-      <c r="I85" s="2"/>
-      <c r="J85" s="2"/>
-      <c r="K85" s="2"/>
-      <c r="L85" s="2"/>
+      <c r="A85" s="66"/>
+      <c r="B85" s="67"/>
+      <c r="C85" s="67"/>
+      <c r="D85" s="72"/>
+      <c r="E85" s="72"/>
+      <c r="F85" s="72"/>
+      <c r="G85" s="72"/>
+      <c r="H85" s="72"/>
+      <c r="I85" s="72"/>
+      <c r="J85" s="137"/>
+      <c r="K85" s="138"/>
+      <c r="L85" s="139"/>
       <c r="M85" s="2"/>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
@@ -6135,18 +6104,18 @@
       <c r="AU85" s="2"/>
     </row>
     <row r="86" spans="1:47" ht="12.75">
-      <c r="A86" s="1"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="2"/>
-      <c r="G86" s="2"/>
-      <c r="H86" s="2"/>
-      <c r="I86" s="2"/>
-      <c r="J86" s="2"/>
-      <c r="K86" s="2"/>
-      <c r="L86" s="2"/>
+      <c r="A86" s="66"/>
+      <c r="B86" s="67"/>
+      <c r="C86" s="67"/>
+      <c r="D86" s="72"/>
+      <c r="E86" s="72"/>
+      <c r="F86" s="72"/>
+      <c r="G86" s="72"/>
+      <c r="H86" s="72"/>
+      <c r="I86" s="72"/>
+      <c r="J86" s="137"/>
+      <c r="K86" s="138"/>
+      <c r="L86" s="139"/>
       <c r="M86" s="2"/>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -6184,18 +6153,23 @@
       <c r="AU86" s="2"/>
     </row>
     <row r="87" spans="1:47" ht="12.75">
-      <c r="A87" s="1"/>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
-      <c r="H87" s="2"/>
-      <c r="I87" s="2"/>
-      <c r="J87" s="2"/>
-      <c r="K87" s="2"/>
-      <c r="L87" s="2"/>
+      <c r="A87" s="66"/>
+      <c r="B87" s="67"/>
+      <c r="C87" s="67"/>
+      <c r="D87" s="84"/>
+      <c r="E87" s="72"/>
+      <c r="F87" s="72"/>
+      <c r="G87" s="72"/>
+      <c r="H87" s="72"/>
+      <c r="I87" s="72"/>
+      <c r="J87" s="85" t="s">
+        <v>100</v>
+      </c>
+      <c r="K87" s="86"/>
+      <c r="L87" s="87">
+        <f>SUM(L19:L68)</f>
+        <v>131155.83000000002</v>
+      </c>
       <c r="M87" s="2"/>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -6232,19 +6206,21 @@
       <c r="AT87" s="2"/>
       <c r="AU87" s="2"/>
     </row>
-    <row r="88" spans="1:47" ht="12.75">
-      <c r="A88" s="1"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
-      <c r="H88" s="2"/>
-      <c r="I88" s="2"/>
-      <c r="J88" s="2"/>
-      <c r="K88" s="2"/>
-      <c r="L88" s="2"/>
+    <row r="88" spans="1:47" ht="14.25">
+      <c r="A88" s="88"/>
+      <c r="B88" s="89"/>
+      <c r="C88" s="89"/>
+      <c r="D88" s="89"/>
+      <c r="E88" s="89"/>
+      <c r="F88" s="90"/>
+      <c r="G88" s="135" t="s">
+        <v>101</v>
+      </c>
+      <c r="H88" s="116"/>
+      <c r="I88" s="116"/>
+      <c r="J88" s="116"/>
+      <c r="K88" s="116"/>
+      <c r="L88" s="117"/>
       <c r="M88" s="2"/>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -6281,21 +6257,625 @@
       <c r="AT88" s="2"/>
       <c r="AU88" s="2"/>
     </row>
+    <row r="89" spans="1:47" ht="14.25">
+      <c r="A89" s="91"/>
+      <c r="B89" s="9"/>
+      <c r="C89" s="9"/>
+      <c r="D89" s="9"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="92"/>
+      <c r="G89" s="9"/>
+      <c r="H89" s="9"/>
+      <c r="I89" s="9"/>
+      <c r="J89" s="9"/>
+      <c r="K89" s="9"/>
+      <c r="L89" s="93"/>
+      <c r="M89" s="2"/>
+      <c r="N89" s="2"/>
+      <c r="O89" s="2"/>
+      <c r="P89" s="2"/>
+      <c r="Q89" s="2"/>
+      <c r="R89" s="2"/>
+      <c r="S89" s="2"/>
+      <c r="T89" s="2"/>
+      <c r="U89" s="2"/>
+      <c r="V89" s="2"/>
+      <c r="W89" s="2"/>
+      <c r="X89" s="2"/>
+      <c r="Y89" s="2"/>
+      <c r="Z89" s="2"/>
+      <c r="AA89" s="2"/>
+      <c r="AB89" s="2"/>
+      <c r="AC89" s="2"/>
+      <c r="AD89" s="2"/>
+      <c r="AE89" s="2"/>
+      <c r="AF89" s="2"/>
+      <c r="AG89" s="2"/>
+      <c r="AH89" s="2"/>
+      <c r="AI89" s="2"/>
+      <c r="AJ89" s="2"/>
+      <c r="AK89" s="2"/>
+      <c r="AL89" s="2"/>
+      <c r="AM89" s="2"/>
+      <c r="AN89" s="2"/>
+      <c r="AO89" s="2"/>
+      <c r="AP89" s="2"/>
+      <c r="AQ89" s="2"/>
+      <c r="AR89" s="2"/>
+      <c r="AS89" s="2"/>
+      <c r="AT89" s="2"/>
+      <c r="AU89" s="2"/>
+    </row>
+    <row r="90" spans="1:47" ht="14.25">
+      <c r="A90" s="94"/>
+      <c r="B90" s="127" t="s">
+        <v>102</v>
+      </c>
+      <c r="C90" s="107"/>
+      <c r="D90" s="9"/>
+      <c r="E90" s="9"/>
+      <c r="F90" s="92"/>
+      <c r="G90" s="9"/>
+      <c r="H90" s="136" t="s">
+        <v>103</v>
+      </c>
+      <c r="I90" s="107"/>
+      <c r="J90" s="9"/>
+      <c r="K90" s="9"/>
+      <c r="L90" s="93"/>
+      <c r="M90" s="2"/>
+      <c r="N90" s="2"/>
+      <c r="O90" s="2"/>
+      <c r="P90" s="2"/>
+      <c r="Q90" s="2"/>
+      <c r="R90" s="2"/>
+      <c r="S90" s="2"/>
+      <c r="T90" s="2"/>
+      <c r="U90" s="2"/>
+      <c r="V90" s="2"/>
+      <c r="W90" s="2"/>
+      <c r="X90" s="2"/>
+      <c r="Y90" s="2"/>
+      <c r="Z90" s="2"/>
+      <c r="AA90" s="2"/>
+      <c r="AB90" s="2"/>
+      <c r="AC90" s="2"/>
+      <c r="AD90" s="2"/>
+      <c r="AE90" s="2"/>
+      <c r="AF90" s="2"/>
+      <c r="AG90" s="2"/>
+      <c r="AH90" s="2"/>
+      <c r="AI90" s="2"/>
+      <c r="AJ90" s="2"/>
+      <c r="AK90" s="2"/>
+      <c r="AL90" s="2"/>
+      <c r="AM90" s="2"/>
+      <c r="AN90" s="2"/>
+      <c r="AO90" s="2"/>
+      <c r="AP90" s="2"/>
+      <c r="AQ90" s="2"/>
+      <c r="AR90" s="2"/>
+      <c r="AS90" s="2"/>
+      <c r="AT90" s="2"/>
+      <c r="AU90" s="2"/>
+    </row>
+    <row r="91" spans="1:47" ht="14.25">
+      <c r="A91" s="94"/>
+      <c r="B91" s="95"/>
+      <c r="C91" s="95"/>
+      <c r="D91" s="9"/>
+      <c r="E91" s="9"/>
+      <c r="F91" s="92"/>
+      <c r="G91" s="9"/>
+      <c r="H91" s="96"/>
+      <c r="I91" s="96"/>
+      <c r="J91" s="9"/>
+      <c r="K91" s="9"/>
+      <c r="L91" s="93"/>
+      <c r="M91" s="2"/>
+      <c r="N91" s="2"/>
+      <c r="O91" s="2"/>
+      <c r="P91" s="2"/>
+      <c r="Q91" s="2"/>
+      <c r="R91" s="2"/>
+      <c r="S91" s="2"/>
+      <c r="T91" s="2"/>
+      <c r="U91" s="2"/>
+      <c r="V91" s="2"/>
+      <c r="W91" s="2"/>
+      <c r="X91" s="2"/>
+      <c r="Y91" s="2"/>
+      <c r="Z91" s="2"/>
+      <c r="AA91" s="2"/>
+      <c r="AB91" s="2"/>
+      <c r="AC91" s="2"/>
+      <c r="AD91" s="2"/>
+      <c r="AE91" s="2"/>
+      <c r="AF91" s="2"/>
+      <c r="AG91" s="2"/>
+      <c r="AH91" s="2"/>
+      <c r="AI91" s="2"/>
+      <c r="AJ91" s="2"/>
+      <c r="AK91" s="2"/>
+      <c r="AL91" s="2"/>
+      <c r="AM91" s="2"/>
+      <c r="AN91" s="2"/>
+      <c r="AO91" s="2"/>
+      <c r="AP91" s="2"/>
+      <c r="AQ91" s="2"/>
+      <c r="AR91" s="2"/>
+      <c r="AS91" s="2"/>
+      <c r="AT91" s="2"/>
+      <c r="AU91" s="2"/>
+    </row>
+    <row r="92" spans="1:47" ht="15">
+      <c r="A92" s="91"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="97" t="s">
+        <v>104</v>
+      </c>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="92"/>
+      <c r="G92" s="9"/>
+      <c r="H92" s="98"/>
+      <c r="I92" s="132" t="s">
+        <v>105</v>
+      </c>
+      <c r="J92" s="107"/>
+      <c r="K92" s="9"/>
+      <c r="L92" s="93"/>
+      <c r="M92" s="2"/>
+      <c r="N92" s="2"/>
+      <c r="O92" s="2"/>
+      <c r="P92" s="2"/>
+      <c r="Q92" s="2"/>
+      <c r="R92" s="2"/>
+      <c r="S92" s="2"/>
+      <c r="T92" s="2"/>
+      <c r="U92" s="2"/>
+      <c r="V92" s="2"/>
+      <c r="W92" s="2"/>
+      <c r="X92" s="2"/>
+      <c r="Y92" s="2"/>
+      <c r="Z92" s="2"/>
+      <c r="AA92" s="2"/>
+      <c r="AB92" s="2"/>
+      <c r="AC92" s="2"/>
+      <c r="AD92" s="2"/>
+      <c r="AE92" s="2"/>
+      <c r="AF92" s="2"/>
+      <c r="AG92" s="2"/>
+      <c r="AH92" s="2"/>
+      <c r="AI92" s="2"/>
+      <c r="AJ92" s="2"/>
+      <c r="AK92" s="2"/>
+      <c r="AL92" s="2"/>
+      <c r="AM92" s="2"/>
+      <c r="AN92" s="2"/>
+      <c r="AO92" s="2"/>
+      <c r="AP92" s="2"/>
+      <c r="AQ92" s="2"/>
+      <c r="AR92" s="2"/>
+      <c r="AS92" s="2"/>
+      <c r="AT92" s="2"/>
+      <c r="AU92" s="2"/>
+    </row>
+    <row r="93" spans="1:47" ht="14.25">
+      <c r="A93" s="91"/>
+      <c r="B93" s="9"/>
+      <c r="C93" s="99" t="s">
+        <v>106</v>
+      </c>
+      <c r="D93" s="9"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="92"/>
+      <c r="G93" s="9"/>
+      <c r="H93" s="9"/>
+      <c r="I93" s="133" t="s">
+        <v>107</v>
+      </c>
+      <c r="J93" s="107"/>
+      <c r="K93" s="9"/>
+      <c r="L93" s="93"/>
+      <c r="M93" s="2"/>
+      <c r="N93" s="2"/>
+      <c r="O93" s="2"/>
+      <c r="P93" s="2"/>
+      <c r="Q93" s="2"/>
+      <c r="R93" s="2"/>
+      <c r="S93" s="2"/>
+      <c r="T93" s="2"/>
+      <c r="U93" s="2"/>
+      <c r="V93" s="2"/>
+      <c r="W93" s="2"/>
+      <c r="X93" s="2"/>
+      <c r="Y93" s="2"/>
+      <c r="Z93" s="2"/>
+      <c r="AA93" s="2"/>
+      <c r="AB93" s="2"/>
+      <c r="AC93" s="2"/>
+      <c r="AD93" s="2"/>
+      <c r="AE93" s="2"/>
+      <c r="AF93" s="2"/>
+      <c r="AG93" s="2"/>
+      <c r="AH93" s="2"/>
+      <c r="AI93" s="2"/>
+      <c r="AJ93" s="2"/>
+      <c r="AK93" s="2"/>
+      <c r="AL93" s="2"/>
+      <c r="AM93" s="2"/>
+      <c r="AN93" s="2"/>
+      <c r="AO93" s="2"/>
+      <c r="AP93" s="2"/>
+      <c r="AQ93" s="2"/>
+      <c r="AR93" s="2"/>
+      <c r="AS93" s="2"/>
+      <c r="AT93" s="2"/>
+      <c r="AU93" s="2"/>
+    </row>
+    <row r="94" spans="1:47" ht="14.25">
+      <c r="A94" s="91"/>
+      <c r="B94" s="9"/>
+      <c r="C94" s="9"/>
+      <c r="D94" s="9"/>
+      <c r="E94" s="9"/>
+      <c r="F94" s="92"/>
+      <c r="G94" s="9"/>
+      <c r="H94" s="9"/>
+      <c r="I94" s="9"/>
+      <c r="J94" s="9"/>
+      <c r="K94" s="9"/>
+      <c r="L94" s="93"/>
+      <c r="M94" s="2"/>
+      <c r="N94" s="2"/>
+      <c r="O94" s="2"/>
+      <c r="P94" s="2"/>
+      <c r="Q94" s="2"/>
+      <c r="R94" s="2"/>
+      <c r="S94" s="2"/>
+      <c r="T94" s="2"/>
+      <c r="U94" s="2"/>
+      <c r="V94" s="2"/>
+      <c r="W94" s="2"/>
+      <c r="X94" s="2"/>
+      <c r="Y94" s="2"/>
+      <c r="Z94" s="2"/>
+      <c r="AA94" s="2"/>
+      <c r="AB94" s="2"/>
+      <c r="AC94" s="2"/>
+      <c r="AD94" s="2"/>
+      <c r="AE94" s="2"/>
+      <c r="AF94" s="2"/>
+      <c r="AG94" s="2"/>
+      <c r="AH94" s="2"/>
+      <c r="AI94" s="2"/>
+      <c r="AJ94" s="2"/>
+      <c r="AK94" s="2"/>
+      <c r="AL94" s="2"/>
+      <c r="AM94" s="2"/>
+      <c r="AN94" s="2"/>
+      <c r="AO94" s="2"/>
+      <c r="AP94" s="2"/>
+      <c r="AQ94" s="2"/>
+      <c r="AR94" s="2"/>
+      <c r="AS94" s="2"/>
+      <c r="AT94" s="2"/>
+      <c r="AU94" s="2"/>
+    </row>
+    <row r="95" spans="1:47" ht="14.25">
+      <c r="A95" s="88"/>
+      <c r="B95" s="89"/>
+      <c r="C95" s="134" t="s">
+        <v>108</v>
+      </c>
+      <c r="D95" s="113"/>
+      <c r="E95" s="113"/>
+      <c r="F95" s="90"/>
+      <c r="G95" s="89"/>
+      <c r="H95" s="89"/>
+      <c r="I95" s="134" t="s">
+        <v>109</v>
+      </c>
+      <c r="J95" s="113"/>
+      <c r="K95" s="89"/>
+      <c r="L95" s="100"/>
+      <c r="M95" s="2"/>
+      <c r="N95" s="2"/>
+      <c r="O95" s="2"/>
+      <c r="P95" s="2"/>
+      <c r="Q95" s="2"/>
+      <c r="R95" s="2"/>
+      <c r="S95" s="2"/>
+      <c r="T95" s="2"/>
+      <c r="U95" s="2"/>
+      <c r="V95" s="2"/>
+      <c r="W95" s="2"/>
+      <c r="X95" s="2"/>
+      <c r="Y95" s="2"/>
+      <c r="Z95" s="2"/>
+      <c r="AA95" s="2"/>
+      <c r="AB95" s="2"/>
+      <c r="AC95" s="2"/>
+      <c r="AD95" s="2"/>
+      <c r="AE95" s="2"/>
+      <c r="AF95" s="2"/>
+      <c r="AG95" s="2"/>
+      <c r="AH95" s="2"/>
+      <c r="AI95" s="2"/>
+      <c r="AJ95" s="2"/>
+      <c r="AK95" s="2"/>
+      <c r="AL95" s="2"/>
+      <c r="AM95" s="2"/>
+      <c r="AN95" s="2"/>
+      <c r="AO95" s="2"/>
+      <c r="AP95" s="2"/>
+      <c r="AQ95" s="2"/>
+      <c r="AR95" s="2"/>
+      <c r="AS95" s="2"/>
+      <c r="AT95" s="2"/>
+      <c r="AU95" s="2"/>
+    </row>
+    <row r="96" spans="1:47" ht="12.75">
+      <c r="A96" s="1"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="E96" s="2"/>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
+      <c r="H96" s="2"/>
+      <c r="I96" s="2"/>
+      <c r="J96" s="2"/>
+      <c r="K96" s="2"/>
+      <c r="L96" s="2"/>
+      <c r="M96" s="2"/>
+      <c r="N96" s="2"/>
+      <c r="O96" s="2"/>
+      <c r="P96" s="2"/>
+      <c r="Q96" s="2"/>
+      <c r="R96" s="2"/>
+      <c r="S96" s="2"/>
+      <c r="T96" s="2"/>
+      <c r="U96" s="2"/>
+      <c r="V96" s="2"/>
+      <c r="W96" s="2"/>
+      <c r="X96" s="2"/>
+      <c r="Y96" s="2"/>
+      <c r="Z96" s="2"/>
+      <c r="AA96" s="2"/>
+      <c r="AB96" s="2"/>
+      <c r="AC96" s="2"/>
+      <c r="AD96" s="2"/>
+      <c r="AE96" s="2"/>
+      <c r="AF96" s="2"/>
+      <c r="AG96" s="2"/>
+      <c r="AH96" s="2"/>
+      <c r="AI96" s="2"/>
+      <c r="AJ96" s="2"/>
+      <c r="AK96" s="2"/>
+      <c r="AL96" s="2"/>
+      <c r="AM96" s="2"/>
+      <c r="AN96" s="2"/>
+      <c r="AO96" s="2"/>
+      <c r="AP96" s="2"/>
+      <c r="AQ96" s="2"/>
+      <c r="AR96" s="2"/>
+      <c r="AS96" s="2"/>
+      <c r="AT96" s="2"/>
+      <c r="AU96" s="2"/>
+    </row>
+    <row r="97" spans="1:47" ht="12.75">
+      <c r="A97" s="1"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2"/>
+      <c r="F97" s="2"/>
+      <c r="G97" s="2"/>
+      <c r="H97" s="2"/>
+      <c r="I97" s="2"/>
+      <c r="J97" s="2"/>
+      <c r="K97" s="2"/>
+      <c r="L97" s="2"/>
+      <c r="M97" s="2"/>
+      <c r="N97" s="2"/>
+      <c r="O97" s="2"/>
+      <c r="P97" s="2"/>
+      <c r="Q97" s="2"/>
+      <c r="R97" s="2"/>
+      <c r="S97" s="2"/>
+      <c r="T97" s="2"/>
+      <c r="U97" s="2"/>
+      <c r="V97" s="2"/>
+      <c r="W97" s="2"/>
+      <c r="X97" s="2"/>
+      <c r="Y97" s="2"/>
+      <c r="Z97" s="2"/>
+      <c r="AA97" s="2"/>
+      <c r="AB97" s="2"/>
+      <c r="AC97" s="2"/>
+      <c r="AD97" s="2"/>
+      <c r="AE97" s="2"/>
+      <c r="AF97" s="2"/>
+      <c r="AG97" s="2"/>
+      <c r="AH97" s="2"/>
+      <c r="AI97" s="2"/>
+      <c r="AJ97" s="2"/>
+      <c r="AK97" s="2"/>
+      <c r="AL97" s="2"/>
+      <c r="AM97" s="2"/>
+      <c r="AN97" s="2"/>
+      <c r="AO97" s="2"/>
+      <c r="AP97" s="2"/>
+      <c r="AQ97" s="2"/>
+      <c r="AR97" s="2"/>
+      <c r="AS97" s="2"/>
+      <c r="AT97" s="2"/>
+      <c r="AU97" s="2"/>
+    </row>
+    <row r="98" spans="1:47" ht="12.75">
+      <c r="A98" s="1"/>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
+      <c r="D98" s="2"/>
+      <c r="E98" s="2"/>
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
+      <c r="H98" s="2"/>
+      <c r="I98" s="2"/>
+      <c r="J98" s="2"/>
+      <c r="K98" s="2"/>
+      <c r="L98" s="2"/>
+      <c r="M98" s="2"/>
+      <c r="N98" s="2"/>
+      <c r="O98" s="2"/>
+      <c r="P98" s="2"/>
+      <c r="Q98" s="2"/>
+      <c r="R98" s="2"/>
+      <c r="S98" s="2"/>
+      <c r="T98" s="2"/>
+      <c r="U98" s="2"/>
+      <c r="V98" s="2"/>
+      <c r="W98" s="2"/>
+      <c r="X98" s="2"/>
+      <c r="Y98" s="2"/>
+      <c r="Z98" s="2"/>
+      <c r="AA98" s="2"/>
+      <c r="AB98" s="2"/>
+      <c r="AC98" s="2"/>
+      <c r="AD98" s="2"/>
+      <c r="AE98" s="2"/>
+      <c r="AF98" s="2"/>
+      <c r="AG98" s="2"/>
+      <c r="AH98" s="2"/>
+      <c r="AI98" s="2"/>
+      <c r="AJ98" s="2"/>
+      <c r="AK98" s="2"/>
+      <c r="AL98" s="2"/>
+      <c r="AM98" s="2"/>
+      <c r="AN98" s="2"/>
+      <c r="AO98" s="2"/>
+      <c r="AP98" s="2"/>
+      <c r="AQ98" s="2"/>
+      <c r="AR98" s="2"/>
+      <c r="AS98" s="2"/>
+      <c r="AT98" s="2"/>
+      <c r="AU98" s="2"/>
+    </row>
+    <row r="99" spans="1:47" ht="12.75">
+      <c r="A99" s="1"/>
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+      <c r="H99" s="2"/>
+      <c r="I99" s="2"/>
+      <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
+      <c r="L99" s="2"/>
+      <c r="M99" s="2"/>
+      <c r="N99" s="2"/>
+      <c r="O99" s="2"/>
+      <c r="P99" s="2"/>
+      <c r="Q99" s="2"/>
+      <c r="R99" s="2"/>
+      <c r="S99" s="2"/>
+      <c r="T99" s="2"/>
+      <c r="U99" s="2"/>
+      <c r="V99" s="2"/>
+      <c r="W99" s="2"/>
+      <c r="X99" s="2"/>
+      <c r="Y99" s="2"/>
+      <c r="Z99" s="2"/>
+      <c r="AA99" s="2"/>
+      <c r="AB99" s="2"/>
+      <c r="AC99" s="2"/>
+      <c r="AD99" s="2"/>
+      <c r="AE99" s="2"/>
+      <c r="AF99" s="2"/>
+      <c r="AG99" s="2"/>
+      <c r="AH99" s="2"/>
+      <c r="AI99" s="2"/>
+      <c r="AJ99" s="2"/>
+      <c r="AK99" s="2"/>
+      <c r="AL99" s="2"/>
+      <c r="AM99" s="2"/>
+      <c r="AN99" s="2"/>
+      <c r="AO99" s="2"/>
+      <c r="AP99" s="2"/>
+      <c r="AQ99" s="2"/>
+      <c r="AR99" s="2"/>
+      <c r="AS99" s="2"/>
+      <c r="AT99" s="2"/>
+      <c r="AU99" s="2"/>
+    </row>
+    <row r="100" spans="1:47" ht="12.75">
+      <c r="A100" s="1"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
+      <c r="H100" s="2"/>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+      <c r="K100" s="2"/>
+      <c r="L100" s="2"/>
+      <c r="M100" s="2"/>
+      <c r="N100" s="2"/>
+      <c r="O100" s="2"/>
+      <c r="P100" s="2"/>
+      <c r="Q100" s="2"/>
+      <c r="R100" s="2"/>
+      <c r="S100" s="2"/>
+      <c r="T100" s="2"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2"/>
+      <c r="W100" s="2"/>
+      <c r="X100" s="2"/>
+      <c r="Y100" s="2"/>
+      <c r="Z100" s="2"/>
+      <c r="AA100" s="2"/>
+      <c r="AB100" s="2"/>
+      <c r="AC100" s="2"/>
+      <c r="AD100" s="2"/>
+      <c r="AE100" s="2"/>
+      <c r="AF100" s="2"/>
+      <c r="AG100" s="2"/>
+      <c r="AH100" s="2"/>
+      <c r="AI100" s="2"/>
+      <c r="AJ100" s="2"/>
+      <c r="AK100" s="2"/>
+      <c r="AL100" s="2"/>
+      <c r="AM100" s="2"/>
+      <c r="AN100" s="2"/>
+      <c r="AO100" s="2"/>
+      <c r="AP100" s="2"/>
+      <c r="AQ100" s="2"/>
+      <c r="AR100" s="2"/>
+      <c r="AS100" s="2"/>
+      <c r="AT100" s="2"/>
+      <c r="AU100" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="I80:J80"/>
-    <mergeCell ref="I81:J81"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="I83:J83"/>
+    <mergeCell ref="I92:J92"/>
+    <mergeCell ref="I93:J93"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="I95:J95"/>
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="I11:L11"/>
     <mergeCell ref="I12:L12"/>
     <mergeCell ref="G14:L15"/>
     <mergeCell ref="J16:L16"/>
-    <mergeCell ref="G76:L76"/>
-    <mergeCell ref="H78:I78"/>
+    <mergeCell ref="G88:L88"/>
+    <mergeCell ref="H90:I90"/>
     <mergeCell ref="C14:C18"/>
-    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B90:C90"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A11:D11"/>
@@ -6323,7 +6903,10 @@
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="5" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
+  <pageSetup paperSize="5" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" fitToWidth="1" fitToHeight="0"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="43" min="0" max="11" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Repair expanded CDR workbook
</commit_message>
<xml_diff>
--- a/assets/cdr_template.xlsx
+++ b/assets/cdr_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jo Ann\Desktop\joannmarie\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jo Ann\dwdatlas\.tmp-cdr-repair\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -16,11 +16,11 @@
     <sheet name="Cabacungan ES-Q2" sheetId="2" r:id="rId2"/>
     <sheet name="UACS" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="152511"/>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabacungan ES-Q1'!$A$1:$L$95</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cabacungan ES-Q1'!$14:$18</definedName>
   </definedNames>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -786,7 +786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1063,6 +1063,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1112,9 +1120,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1138,12 +1143,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1380,36 +1381,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:47" ht="16.5">
-      <c r="A2" s="106" t="s">
+      <c r="A2" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="107"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
+      <c r="B2" s="111"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
     </row>
     <row r="3" spans="1:47" ht="16.5">
-      <c r="A3" s="108" t="s">
+      <c r="A3" s="112" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="107"/>
-      <c r="C3" s="107"/>
-      <c r="D3" s="107"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="107"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="107"/>
-      <c r="L3" s="107"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
     </row>
     <row r="4" spans="1:47" ht="18.75">
       <c r="A4" s="1"/>
@@ -1421,11 +1422,11 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="109" t="s">
+      <c r="J4" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="107"/>
-      <c r="L4" s="107"/>
+      <c r="K4" s="111"/>
+      <c r="L4" s="111"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1512,20 +1513,20 @@
       <c r="AU5" s="2"/>
     </row>
     <row r="6" spans="1:47" ht="18">
-      <c r="A6" s="110" t="s">
+      <c r="A6" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="107"/>
-      <c r="C6" s="107"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="107"/>
-      <c r="I6" s="107"/>
-      <c r="J6" s="107"/>
-      <c r="K6" s="107"/>
-      <c r="L6" s="107"/>
+      <c r="B6" s="111"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="111"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="111"/>
+      <c r="L6" s="111"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -1612,22 +1613,22 @@
       <c r="AU7" s="4"/>
     </row>
     <row r="8" spans="1:47" ht="18">
-      <c r="A8" s="111" t="s">
+      <c r="A8" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="107"/>
-      <c r="C8" s="107"/>
-      <c r="D8" s="107"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
       <c r="E8" s="7"/>
       <c r="F8" s="5"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="111" t="s">
+      <c r="I8" s="115" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="107"/>
-      <c r="K8" s="107"/>
-      <c r="L8" s="107"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="111"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
@@ -1665,22 +1666,22 @@
       <c r="AU8" s="4"/>
     </row>
     <row r="9" spans="1:47" ht="18">
-      <c r="A9" s="111" t="s">
+      <c r="A9" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="107"/>
-      <c r="C9" s="107"/>
-      <c r="D9" s="107"/>
+      <c r="B9" s="111"/>
+      <c r="C9" s="111"/>
+      <c r="D9" s="111"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="111" t="s">
+      <c r="I9" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="107"/>
-      <c r="K9" s="107"/>
-      <c r="L9" s="107"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="111"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
@@ -1718,22 +1719,22 @@
       <c r="AU9" s="4"/>
     </row>
     <row r="10" spans="1:47" ht="18">
-      <c r="A10" s="111" t="s">
+      <c r="A10" s="115" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="107"/>
-      <c r="C10" s="107"/>
-      <c r="D10" s="107"/>
+      <c r="B10" s="111"/>
+      <c r="C10" s="111"/>
+      <c r="D10" s="111"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="111" t="s">
+      <c r="I10" s="115" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="107"/>
-      <c r="K10" s="107"/>
-      <c r="L10" s="107"/>
+      <c r="J10" s="111"/>
+      <c r="K10" s="111"/>
+      <c r="L10" s="111"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
@@ -1771,22 +1772,22 @@
       <c r="AU10" s="4"/>
     </row>
     <row r="11" spans="1:47" ht="18">
-      <c r="A11" s="111" t="s">
+      <c r="A11" s="115" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="107"/>
-      <c r="C11" s="107"/>
-      <c r="D11" s="107"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="111"/>
+      <c r="D11" s="111"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
-      <c r="I11" s="111" t="s">
+      <c r="I11" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="107"/>
-      <c r="K11" s="107"/>
-      <c r="L11" s="107"/>
+      <c r="J11" s="111"/>
+      <c r="K11" s="111"/>
+      <c r="L11" s="111"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
@@ -1832,12 +1833,12 @@
       <c r="F12" s="5"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="111" t="s">
+      <c r="I12" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="107"/>
-      <c r="K12" s="107"/>
-      <c r="L12" s="107"/>
+      <c r="J12" s="111"/>
+      <c r="K12" s="111"/>
+      <c r="L12" s="111"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
@@ -1924,28 +1925,28 @@
       <c r="AU13" s="4"/>
     </row>
     <row r="14" spans="1:47" ht="18">
-      <c r="A14" s="125" t="s">
+      <c r="A14" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="128" t="s">
+      <c r="B14" s="131" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="125" t="s">
+      <c r="C14" s="129" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="129" t="s">
+      <c r="D14" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="130"/>
-      <c r="F14" s="131"/>
-      <c r="G14" s="129" t="s">
+      <c r="E14" s="133"/>
+      <c r="F14" s="134"/>
+      <c r="G14" s="132" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="130"/>
-      <c r="I14" s="130"/>
-      <c r="J14" s="130"/>
-      <c r="K14" s="130"/>
-      <c r="L14" s="131"/>
+      <c r="H14" s="133"/>
+      <c r="I14" s="133"/>
+      <c r="J14" s="133"/>
+      <c r="K14" s="133"/>
+      <c r="L14" s="134"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
@@ -1983,20 +1984,20 @@
       <c r="AU14" s="4"/>
     </row>
     <row r="15" spans="1:47" ht="14.25">
-      <c r="A15" s="126"/>
-      <c r="B15" s="126"/>
-      <c r="C15" s="126"/>
-      <c r="D15" s="112">
+      <c r="A15" s="130"/>
+      <c r="B15" s="130"/>
+      <c r="C15" s="130"/>
+      <c r="D15" s="116">
         <v>-19901010</v>
       </c>
-      <c r="E15" s="113"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="113"/>
-      <c r="H15" s="113"/>
-      <c r="I15" s="113"/>
-      <c r="J15" s="113"/>
-      <c r="K15" s="113"/>
-      <c r="L15" s="114"/>
+      <c r="E15" s="117"/>
+      <c r="F15" s="118"/>
+      <c r="G15" s="117"/>
+      <c r="H15" s="117"/>
+      <c r="I15" s="117"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="117"/>
+      <c r="L15" s="118"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
@@ -2034,28 +2035,28 @@
       <c r="AU15" s="10"/>
     </row>
     <row r="16" spans="1:47" ht="14.25">
-      <c r="A16" s="126"/>
-      <c r="B16" s="126"/>
-      <c r="C16" s="126"/>
-      <c r="D16" s="115" t="s">
+      <c r="A16" s="130"/>
+      <c r="B16" s="130"/>
+      <c r="C16" s="130"/>
+      <c r="D16" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="116"/>
-      <c r="F16" s="117"/>
-      <c r="G16" s="118" t="s">
+      <c r="E16" s="120"/>
+      <c r="F16" s="121"/>
+      <c r="G16" s="122" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="119" t="s">
+      <c r="H16" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="118" t="s">
+      <c r="I16" s="122" t="s">
         <v>21</v>
       </c>
-      <c r="J16" s="115" t="s">
+      <c r="J16" s="119" t="s">
         <v>22</v>
       </c>
-      <c r="K16" s="116"/>
-      <c r="L16" s="117"/>
+      <c r="K16" s="120"/>
+      <c r="L16" s="121"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2093,28 +2094,28 @@
       <c r="AU16" s="2"/>
     </row>
     <row r="17" spans="1:47" ht="12.75">
-      <c r="A17" s="126"/>
-      <c r="B17" s="126"/>
-      <c r="C17" s="126"/>
-      <c r="D17" s="121" t="s">
+      <c r="A17" s="130"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="130"/>
+      <c r="D17" s="125" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="122" t="s">
+      <c r="E17" s="126" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="124" t="s">
+      <c r="F17" s="128" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="114"/>
-      <c r="H17" s="120"/>
-      <c r="I17" s="114"/>
-      <c r="J17" s="119" t="s">
+      <c r="G17" s="118"/>
+      <c r="H17" s="124"/>
+      <c r="I17" s="118"/>
+      <c r="J17" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="123" t="s">
+      <c r="K17" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="L17" s="124" t="s">
+      <c r="L17" s="128" t="s">
         <v>18</v>
       </c>
       <c r="M17" s="2"/>
@@ -2154,12 +2155,12 @@
       <c r="AU17" s="2"/>
     </row>
     <row r="18" spans="1:47" ht="12.75">
-      <c r="A18" s="120"/>
-      <c r="B18" s="120"/>
-      <c r="C18" s="120"/>
-      <c r="D18" s="120"/>
-      <c r="E18" s="120"/>
-      <c r="F18" s="114"/>
+      <c r="A18" s="124"/>
+      <c r="B18" s="124"/>
+      <c r="C18" s="124"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="118"/>
       <c r="G18" s="11">
         <v>5020301000</v>
       </c>
@@ -2169,9 +2170,9 @@
       <c r="I18" s="11">
         <v>5021202000</v>
       </c>
-      <c r="J18" s="120"/>
-      <c r="K18" s="120"/>
-      <c r="L18" s="114"/>
+      <c r="J18" s="124"/>
+      <c r="K18" s="124"/>
+      <c r="L18" s="118"/>
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
@@ -4610,18 +4611,19 @@
       <c r="AT56" s="2"/>
       <c r="AU56" s="2"/>
     </row>
-    <row r="57" spans="1:47" ht="25.5">
+    <row r="57" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A57" s="51"/>
       <c r="B57" s="65"/>
       <c r="C57" s="53"/>
       <c r="D57" s="59"/>
+      <c r="E57" s="42"/>
       <c r="F57" s="26"/>
-      <c r="G57" s="32"/>
+      <c r="G57" s="42"/>
       <c r="H57" s="42"/>
       <c r="I57" s="42"/>
       <c r="J57" s="28"/>
-      <c r="K57" s="29"/>
-      <c r="L57" s="32"/>
+      <c r="K57" s="63"/>
+      <c r="L57" s="42"/>
       <c r="M57" s="2"/>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -4658,18 +4660,19 @@
       <c r="AT57" s="2"/>
       <c r="AU57" s="2"/>
     </row>
-    <row r="58" spans="1:47" ht="25.5">
+    <row r="58" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A58" s="51"/>
       <c r="B58" s="65"/>
       <c r="C58" s="53"/>
       <c r="D58" s="59"/>
+      <c r="E58" s="42"/>
       <c r="F58" s="26"/>
-      <c r="G58" s="32"/>
+      <c r="G58" s="42"/>
       <c r="H58" s="42"/>
       <c r="I58" s="42"/>
       <c r="J58" s="28"/>
-      <c r="K58" s="29"/>
-      <c r="L58" s="32"/>
+      <c r="K58" s="63"/>
+      <c r="L58" s="42"/>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -4706,18 +4709,19 @@
       <c r="AT58" s="2"/>
       <c r="AU58" s="2"/>
     </row>
-    <row r="59" spans="1:47" ht="25.5">
+    <row r="59" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A59" s="51"/>
       <c r="B59" s="65"/>
       <c r="C59" s="53"/>
       <c r="D59" s="59"/>
+      <c r="E59" s="42"/>
       <c r="F59" s="26"/>
-      <c r="G59" s="32"/>
+      <c r="G59" s="42"/>
       <c r="H59" s="42"/>
       <c r="I59" s="42"/>
       <c r="J59" s="28"/>
-      <c r="K59" s="29"/>
-      <c r="L59" s="32"/>
+      <c r="K59" s="63"/>
+      <c r="L59" s="42"/>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -4754,18 +4758,19 @@
       <c r="AT59" s="2"/>
       <c r="AU59" s="2"/>
     </row>
-    <row r="60" spans="1:47" ht="25.5">
+    <row r="60" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A60" s="51"/>
       <c r="B60" s="65"/>
       <c r="C60" s="53"/>
       <c r="D60" s="59"/>
+      <c r="E60" s="42"/>
       <c r="F60" s="26"/>
-      <c r="G60" s="32"/>
+      <c r="G60" s="42"/>
       <c r="H60" s="42"/>
       <c r="I60" s="42"/>
       <c r="J60" s="28"/>
-      <c r="K60" s="29"/>
-      <c r="L60" s="32"/>
+      <c r="K60" s="63"/>
+      <c r="L60" s="42"/>
       <c r="M60" s="2"/>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -4802,18 +4807,19 @@
       <c r="AT60" s="2"/>
       <c r="AU60" s="2"/>
     </row>
-    <row r="61" spans="1:47" ht="25.5">
+    <row r="61" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A61" s="51"/>
       <c r="B61" s="65"/>
       <c r="C61" s="53"/>
       <c r="D61" s="59"/>
+      <c r="E61" s="42"/>
       <c r="F61" s="26"/>
-      <c r="G61" s="32"/>
+      <c r="G61" s="42"/>
       <c r="H61" s="42"/>
       <c r="I61" s="42"/>
       <c r="J61" s="28"/>
-      <c r="K61" s="29"/>
-      <c r="L61" s="32"/>
+      <c r="K61" s="63"/>
+      <c r="L61" s="42"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
@@ -4850,18 +4856,19 @@
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
     </row>
-    <row r="62" spans="1:47" ht="25.5">
+    <row r="62" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A62" s="51"/>
       <c r="B62" s="65"/>
       <c r="C62" s="53"/>
       <c r="D62" s="59"/>
+      <c r="E62" s="42"/>
       <c r="F62" s="26"/>
-      <c r="G62" s="32"/>
+      <c r="G62" s="42"/>
       <c r="H62" s="42"/>
       <c r="I62" s="42"/>
       <c r="J62" s="28"/>
-      <c r="K62" s="29"/>
-      <c r="L62" s="32"/>
+      <c r="K62" s="63"/>
+      <c r="L62" s="42"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -4898,18 +4905,19 @@
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
     </row>
-    <row r="63" spans="1:47" ht="25.5">
+    <row r="63" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A63" s="51"/>
       <c r="B63" s="65"/>
       <c r="C63" s="53"/>
       <c r="D63" s="59"/>
+      <c r="E63" s="42"/>
       <c r="F63" s="26"/>
-      <c r="G63" s="32"/>
+      <c r="G63" s="42"/>
       <c r="H63" s="42"/>
       <c r="I63" s="42"/>
       <c r="J63" s="28"/>
-      <c r="K63" s="29"/>
-      <c r="L63" s="32"/>
+      <c r="K63" s="63"/>
+      <c r="L63" s="42"/>
       <c r="M63" s="2"/>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -4946,18 +4954,19 @@
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
     </row>
-    <row r="64" spans="1:47" ht="25.5">
+    <row r="64" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A64" s="51"/>
       <c r="B64" s="65"/>
       <c r="C64" s="53"/>
       <c r="D64" s="59"/>
+      <c r="E64" s="42"/>
       <c r="F64" s="26"/>
-      <c r="G64" s="32"/>
+      <c r="G64" s="42"/>
       <c r="H64" s="42"/>
       <c r="I64" s="42"/>
       <c r="J64" s="28"/>
-      <c r="K64" s="29"/>
-      <c r="L64" s="32"/>
+      <c r="K64" s="63"/>
+      <c r="L64" s="42"/>
       <c r="M64" s="2"/>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -4994,18 +5003,19 @@
       <c r="AT64" s="2"/>
       <c r="AU64" s="2"/>
     </row>
-    <row r="65" spans="1:47" ht="25.5">
+    <row r="65" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A65" s="51"/>
       <c r="B65" s="65"/>
       <c r="C65" s="53"/>
       <c r="D65" s="59"/>
+      <c r="E65" s="42"/>
       <c r="F65" s="26"/>
-      <c r="G65" s="32"/>
+      <c r="G65" s="42"/>
       <c r="H65" s="42"/>
       <c r="I65" s="42"/>
       <c r="J65" s="28"/>
-      <c r="K65" s="29"/>
-      <c r="L65" s="32"/>
+      <c r="K65" s="63"/>
+      <c r="L65" s="42"/>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -5042,18 +5052,19 @@
       <c r="AT65" s="2"/>
       <c r="AU65" s="2"/>
     </row>
-    <row r="66" spans="1:47" ht="25.5">
+    <row r="66" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A66" s="51"/>
       <c r="B66" s="65"/>
       <c r="C66" s="53"/>
       <c r="D66" s="59"/>
+      <c r="E66" s="42"/>
       <c r="F66" s="26"/>
-      <c r="G66" s="32"/>
+      <c r="G66" s="42"/>
       <c r="H66" s="42"/>
       <c r="I66" s="42"/>
       <c r="J66" s="28"/>
-      <c r="K66" s="29"/>
-      <c r="L66" s="32"/>
+      <c r="K66" s="63"/>
+      <c r="L66" s="42"/>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -5090,18 +5101,19 @@
       <c r="AT66" s="2"/>
       <c r="AU66" s="2"/>
     </row>
-    <row r="67" spans="1:47" ht="25.5">
+    <row r="67" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A67" s="51"/>
       <c r="B67" s="65"/>
       <c r="C67" s="53"/>
       <c r="D67" s="59"/>
+      <c r="E67" s="42"/>
       <c r="F67" s="26"/>
-      <c r="G67" s="32"/>
+      <c r="G67" s="42"/>
       <c r="H67" s="42"/>
       <c r="I67" s="42"/>
       <c r="J67" s="28"/>
-      <c r="K67" s="29"/>
-      <c r="L67" s="32"/>
+      <c r="K67" s="63"/>
+      <c r="L67" s="42"/>
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
@@ -5138,18 +5150,19 @@
       <c r="AT67" s="2"/>
       <c r="AU67" s="2"/>
     </row>
-    <row r="68" spans="1:47" ht="25.5">
+    <row r="68" spans="1:47" s="106" customFormat="1" ht="25.5" customHeight="1">
       <c r="A68" s="51"/>
       <c r="B68" s="65"/>
       <c r="C68" s="53"/>
       <c r="D68" s="59"/>
+      <c r="E68" s="42"/>
       <c r="F68" s="26"/>
-      <c r="G68" s="32"/>
+      <c r="G68" s="42"/>
       <c r="H68" s="42"/>
       <c r="I68" s="42"/>
       <c r="J68" s="28"/>
-      <c r="K68" s="29"/>
-      <c r="L68" s="32"/>
+      <c r="K68" s="63"/>
+      <c r="L68" s="42"/>
       <c r="M68" s="2"/>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -5196,21 +5209,21 @@
       <c r="E69" s="69"/>
       <c r="F69" s="69"/>
       <c r="G69" s="70">
-        <f t="shared" ref="G57:I57" si="1">SUM(G20:G68)</f>
+        <f>SUM(G20:G68)</f>
         <v>60594.17</v>
       </c>
       <c r="H69" s="70">
-        <f t="shared" si="1"/>
+        <f>SUM(H20:H68)</f>
         <v>41000</v>
       </c>
-      <c r="I81" s="70">
-        <f t="shared" si="1"/>
+      <c r="I69" s="70">
+        <f>SUM(I20:I68)</f>
         <v>21000</v>
       </c>
-      <c r="J81" s="71"/>
-      <c r="K81" s="70"/>
-      <c r="L81" s="70">
-        <f>SUM(L19:L68)</f>
+      <c r="J69" s="71"/>
+      <c r="K69" s="70"/>
+      <c r="L69" s="70">
+        <f>SUM(L21:L68)</f>
         <v>131155.83000000002</v>
       </c>
       <c r="M69" s="2"/>
@@ -5533,7 +5546,7 @@
         <v>5020101000</v>
       </c>
       <c r="L75" s="32">
-        <f>SUMIF(J19:J68, "Travelling Expenses-Local", L19:L68)</f>
+        <f>SUMIF(J9:J70, "Travelling Expenses-Local", L9:L70)</f>
         <v>3760</v>
       </c>
       <c r="M75" s="2"/>
@@ -5589,7 +5602,7 @@
         <v>5020502001</v>
       </c>
       <c r="L76" s="32">
-        <f>SUMIF(J19:J68, "Accountable Forms", L19:L68)</f>
+        <f>SUMIF(J1:J70, "Accountable Forms", L1:L70)</f>
         <v>1200</v>
       </c>
       <c r="M76" s="2"/>
@@ -5645,7 +5658,7 @@
         <v>5029902000</v>
       </c>
       <c r="L77" s="32">
-        <f>SUMIF(J19:J68, "Printing and Publication Expenses", L19:L68)</f>
+        <f>SUMIF(J1:J70, "Printing and Publication Expenses", L1:L70)</f>
         <v>3020</v>
       </c>
       <c r="M77" s="2"/>
@@ -5701,7 +5714,7 @@
         <v>5020399000</v>
       </c>
       <c r="L78" s="32">
-        <f>SUMIF(J19:J68, "Other Supplies and Materials Expenses", L19:L68)</f>
+        <f>SUMIF(J1:J70, "Other Supplies and Materials Expenses", L1:L70)</f>
         <v>72498</v>
       </c>
       <c r="M78" s="2"/>
@@ -5757,7 +5770,7 @@
         <v>5021305002</v>
       </c>
       <c r="L79" s="32">
-        <f>SUMIF(J19:J68, "Repairs and Maintenance-Office Equipment", L19:L68)</f>
+        <f>SUMIF(J2:J71, "Repairs and Maintenance-Office Equipment", L2:L71)</f>
         <v>3850</v>
       </c>
       <c r="M79" s="2"/>
@@ -5813,7 +5826,7 @@
         <v>5020201000</v>
       </c>
       <c r="L80" s="32">
-        <f>SUMIF(J19:J68, "Training Expenses", L19:L68)</f>
+        <f>SUMIF(J3:J72, "Training Expenses", L3:L72)</f>
         <v>2990</v>
       </c>
       <c r="M80" s="2"/>
@@ -5917,9 +5930,9 @@
       <c r="G82" s="72"/>
       <c r="H82" s="72"/>
       <c r="I82" s="72"/>
-      <c r="J82" s="137"/>
-      <c r="K82" s="138"/>
-      <c r="L82" s="139"/>
+      <c r="J82" s="107"/>
+      <c r="K82" s="108"/>
+      <c r="L82" s="109"/>
       <c r="M82" s="2"/>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -5966,9 +5979,9 @@
       <c r="G83" s="72"/>
       <c r="H83" s="72"/>
       <c r="I83" s="72"/>
-      <c r="J83" s="137"/>
-      <c r="K83" s="138"/>
-      <c r="L83" s="139"/>
+      <c r="J83" s="107"/>
+      <c r="K83" s="108"/>
+      <c r="L83" s="109"/>
       <c r="M83" s="2"/>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -6015,9 +6028,9 @@
       <c r="G84" s="72"/>
       <c r="H84" s="72"/>
       <c r="I84" s="72"/>
-      <c r="J84" s="137"/>
-      <c r="K84" s="138"/>
-      <c r="L84" s="139"/>
+      <c r="J84" s="107"/>
+      <c r="K84" s="108"/>
+      <c r="L84" s="109"/>
       <c r="M84" s="2"/>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -6064,9 +6077,9 @@
       <c r="G85" s="72"/>
       <c r="H85" s="72"/>
       <c r="I85" s="72"/>
-      <c r="J85" s="137"/>
-      <c r="K85" s="138"/>
-      <c r="L85" s="139"/>
+      <c r="J85" s="107"/>
+      <c r="K85" s="108"/>
+      <c r="L85" s="109"/>
       <c r="M85" s="2"/>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
@@ -6113,9 +6126,9 @@
       <c r="G86" s="72"/>
       <c r="H86" s="72"/>
       <c r="I86" s="72"/>
-      <c r="J86" s="137"/>
-      <c r="K86" s="138"/>
-      <c r="L86" s="139"/>
+      <c r="J86" s="107"/>
+      <c r="K86" s="108"/>
+      <c r="L86" s="109"/>
       <c r="M86" s="2"/>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -6167,7 +6180,7 @@
       </c>
       <c r="K87" s="86"/>
       <c r="L87" s="87">
-        <f>SUM(L19:L68)</f>
+        <f>SUM(L73:L81)</f>
         <v>131155.83000000002</v>
       </c>
       <c r="M87" s="2"/>
@@ -6213,14 +6226,14 @@
       <c r="D88" s="89"/>
       <c r="E88" s="89"/>
       <c r="F88" s="90"/>
-      <c r="G88" s="135" t="s">
+      <c r="G88" s="138" t="s">
         <v>101</v>
       </c>
-      <c r="H88" s="116"/>
-      <c r="I88" s="116"/>
-      <c r="J88" s="116"/>
-      <c r="K88" s="116"/>
-      <c r="L88" s="117"/>
+      <c r="H88" s="120"/>
+      <c r="I88" s="120"/>
+      <c r="J88" s="120"/>
+      <c r="K88" s="120"/>
+      <c r="L88" s="121"/>
       <c r="M88" s="2"/>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -6308,18 +6321,18 @@
     </row>
     <row r="90" spans="1:47" ht="14.25">
       <c r="A90" s="94"/>
-      <c r="B90" s="127" t="s">
+      <c r="B90" s="140" t="s">
         <v>102</v>
       </c>
-      <c r="C90" s="107"/>
+      <c r="C90" s="111"/>
       <c r="D90" s="9"/>
       <c r="E90" s="9"/>
       <c r="F90" s="92"/>
       <c r="G90" s="9"/>
-      <c r="H90" s="136" t="s">
+      <c r="H90" s="139" t="s">
         <v>103</v>
       </c>
-      <c r="I90" s="107"/>
+      <c r="I90" s="111"/>
       <c r="J90" s="9"/>
       <c r="K90" s="9"/>
       <c r="L90" s="93"/>
@@ -6419,10 +6432,10 @@
       <c r="F92" s="92"/>
       <c r="G92" s="9"/>
       <c r="H92" s="98"/>
-      <c r="I92" s="132" t="s">
+      <c r="I92" s="135" t="s">
         <v>105</v>
       </c>
-      <c r="J92" s="107"/>
+      <c r="J92" s="111"/>
       <c r="K92" s="9"/>
       <c r="L92" s="93"/>
       <c r="M92" s="2"/>
@@ -6472,10 +6485,10 @@
       <c r="F93" s="92"/>
       <c r="G93" s="9"/>
       <c r="H93" s="9"/>
-      <c r="I93" s="133" t="s">
+      <c r="I93" s="136" t="s">
         <v>107</v>
       </c>
-      <c r="J93" s="107"/>
+      <c r="J93" s="111"/>
       <c r="K93" s="9"/>
       <c r="L93" s="93"/>
       <c r="M93" s="2"/>
@@ -6566,18 +6579,18 @@
     <row r="95" spans="1:47" ht="14.25">
       <c r="A95" s="88"/>
       <c r="B95" s="89"/>
-      <c r="C95" s="134" t="s">
+      <c r="C95" s="137" t="s">
         <v>108</v>
       </c>
-      <c r="D95" s="113"/>
-      <c r="E95" s="113"/>
+      <c r="D95" s="117"/>
+      <c r="E95" s="117"/>
       <c r="F95" s="90"/>
       <c r="G95" s="89"/>
       <c r="H95" s="89"/>
-      <c r="I95" s="134" t="s">
+      <c r="I95" s="137" t="s">
         <v>109</v>
       </c>
-      <c r="J95" s="113"/>
+      <c r="J95" s="117"/>
       <c r="K95" s="89"/>
       <c r="L95" s="100"/>
       <c r="M95" s="2"/>
@@ -6863,26 +6876,21 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="I92:J92"/>
-    <mergeCell ref="I93:J93"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="I95:J95"/>
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="I11:L11"/>
     <mergeCell ref="I12:L12"/>
     <mergeCell ref="G14:L15"/>
     <mergeCell ref="J16:L16"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="I92:J92"/>
+    <mergeCell ref="I93:J93"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="I95:J95"/>
     <mergeCell ref="G88:L88"/>
     <mergeCell ref="H90:I90"/>
     <mergeCell ref="C14:C18"/>
     <mergeCell ref="B90:C90"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="F17:F18"/>
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
@@ -6894,6 +6902,11 @@
     <mergeCell ref="J17:J18"/>
     <mergeCell ref="K17:K18"/>
     <mergeCell ref="L17:L18"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="J4:L4"/>
@@ -6903,9 +6916,9 @@
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="5" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="5" scale="84" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="43" min="0" max="11" man="1"/>
+    <brk id="43" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
@@ -6928,36 +6941,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:47" ht="16.5">
-      <c r="A2" s="106" t="s">
+      <c r="A2" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="107"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
+      <c r="B2" s="111"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
     </row>
     <row r="3" spans="1:47" ht="16.5">
-      <c r="A3" s="108" t="s">
+      <c r="A3" s="112" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="107"/>
-      <c r="C3" s="107"/>
-      <c r="D3" s="107"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="107"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="107"/>
-      <c r="L3" s="107"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
     </row>
     <row r="4" spans="1:47" ht="18.75">
       <c r="A4" s="1"/>
@@ -6969,11 +6982,11 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="109" t="s">
+      <c r="J4" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="107"/>
-      <c r="L4" s="107"/>
+      <c r="K4" s="111"/>
+      <c r="L4" s="111"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -7060,20 +7073,20 @@
       <c r="AU5" s="2"/>
     </row>
     <row r="6" spans="1:47" ht="18">
-      <c r="A6" s="110" t="s">
+      <c r="A6" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="107"/>
-      <c r="C6" s="107"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="107"/>
-      <c r="I6" s="107"/>
-      <c r="J6" s="107"/>
-      <c r="K6" s="107"/>
-      <c r="L6" s="107"/>
+      <c r="B6" s="111"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="111"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="111"/>
+      <c r="L6" s="111"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -7160,22 +7173,22 @@
       <c r="AU7" s="4"/>
     </row>
     <row r="8" spans="1:47" ht="18">
-      <c r="A8" s="111" t="s">
+      <c r="A8" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="107"/>
-      <c r="C8" s="107"/>
-      <c r="D8" s="107"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
       <c r="E8" s="7"/>
       <c r="F8" s="5"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="111" t="s">
+      <c r="I8" s="115" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="107"/>
-      <c r="K8" s="107"/>
-      <c r="L8" s="107"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="111"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
@@ -7213,22 +7226,22 @@
       <c r="AU8" s="4"/>
     </row>
     <row r="9" spans="1:47" ht="18">
-      <c r="A9" s="111" t="s">
+      <c r="A9" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="107"/>
-      <c r="C9" s="107"/>
-      <c r="D9" s="107"/>
+      <c r="B9" s="111"/>
+      <c r="C9" s="111"/>
+      <c r="D9" s="111"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="111" t="s">
+      <c r="I9" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="107"/>
-      <c r="K9" s="107"/>
-      <c r="L9" s="107"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="111"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
@@ -7266,22 +7279,22 @@
       <c r="AU9" s="4"/>
     </row>
     <row r="10" spans="1:47" ht="18">
-      <c r="A10" s="111" t="s">
+      <c r="A10" s="115" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="107"/>
-      <c r="C10" s="107"/>
-      <c r="D10" s="107"/>
+      <c r="B10" s="111"/>
+      <c r="C10" s="111"/>
+      <c r="D10" s="111"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="111" t="s">
+      <c r="I10" s="115" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="107"/>
-      <c r="K10" s="107"/>
-      <c r="L10" s="107"/>
+      <c r="J10" s="111"/>
+      <c r="K10" s="111"/>
+      <c r="L10" s="111"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
@@ -7319,22 +7332,22 @@
       <c r="AU10" s="4"/>
     </row>
     <row r="11" spans="1:47" ht="18">
-      <c r="A11" s="111" t="s">
+      <c r="A11" s="115" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="107"/>
-      <c r="C11" s="107"/>
-      <c r="D11" s="107"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="111"/>
+      <c r="D11" s="111"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
-      <c r="I11" s="111" t="s">
+      <c r="I11" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="107"/>
-      <c r="K11" s="107"/>
-      <c r="L11" s="107"/>
+      <c r="J11" s="111"/>
+      <c r="K11" s="111"/>
+      <c r="L11" s="111"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
@@ -7380,12 +7393,12 @@
       <c r="F12" s="5"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="111" t="s">
+      <c r="I12" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="107"/>
-      <c r="K12" s="107"/>
-      <c r="L12" s="107"/>
+      <c r="J12" s="111"/>
+      <c r="K12" s="111"/>
+      <c r="L12" s="111"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
@@ -7472,28 +7485,28 @@
       <c r="AU13" s="4"/>
     </row>
     <row r="14" spans="1:47" ht="18">
-      <c r="A14" s="125" t="s">
+      <c r="A14" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="128" t="s">
+      <c r="B14" s="131" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="125" t="s">
+      <c r="C14" s="129" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="129" t="s">
+      <c r="D14" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="130"/>
-      <c r="F14" s="131"/>
-      <c r="G14" s="129" t="s">
+      <c r="E14" s="133"/>
+      <c r="F14" s="134"/>
+      <c r="G14" s="132" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="130"/>
-      <c r="I14" s="130"/>
-      <c r="J14" s="130"/>
-      <c r="K14" s="130"/>
-      <c r="L14" s="131"/>
+      <c r="H14" s="133"/>
+      <c r="I14" s="133"/>
+      <c r="J14" s="133"/>
+      <c r="K14" s="133"/>
+      <c r="L14" s="134"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
@@ -7531,20 +7544,20 @@
       <c r="AU14" s="4"/>
     </row>
     <row r="15" spans="1:47" ht="14.25">
-      <c r="A15" s="126"/>
-      <c r="B15" s="126"/>
-      <c r="C15" s="126"/>
-      <c r="D15" s="112">
+      <c r="A15" s="130"/>
+      <c r="B15" s="130"/>
+      <c r="C15" s="130"/>
+      <c r="D15" s="116">
         <v>-19901010</v>
       </c>
-      <c r="E15" s="113"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="113"/>
-      <c r="H15" s="113"/>
-      <c r="I15" s="113"/>
-      <c r="J15" s="113"/>
-      <c r="K15" s="113"/>
-      <c r="L15" s="114"/>
+      <c r="E15" s="117"/>
+      <c r="F15" s="118"/>
+      <c r="G15" s="117"/>
+      <c r="H15" s="117"/>
+      <c r="I15" s="117"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="117"/>
+      <c r="L15" s="118"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
@@ -7582,28 +7595,28 @@
       <c r="AU15" s="10"/>
     </row>
     <row r="16" spans="1:47" ht="14.25">
-      <c r="A16" s="126"/>
-      <c r="B16" s="126"/>
-      <c r="C16" s="126"/>
-      <c r="D16" s="115" t="s">
+      <c r="A16" s="130"/>
+      <c r="B16" s="130"/>
+      <c r="C16" s="130"/>
+      <c r="D16" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="116"/>
-      <c r="F16" s="117"/>
-      <c r="G16" s="118" t="s">
+      <c r="E16" s="120"/>
+      <c r="F16" s="121"/>
+      <c r="G16" s="122" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="119" t="s">
+      <c r="H16" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="118" t="s">
+      <c r="I16" s="122" t="s">
         <v>21</v>
       </c>
-      <c r="J16" s="115" t="s">
+      <c r="J16" s="119" t="s">
         <v>22</v>
       </c>
-      <c r="K16" s="116"/>
-      <c r="L16" s="117"/>
+      <c r="K16" s="120"/>
+      <c r="L16" s="121"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -7641,28 +7654,28 @@
       <c r="AU16" s="2"/>
     </row>
     <row r="17" spans="1:47" ht="12.75">
-      <c r="A17" s="126"/>
-      <c r="B17" s="126"/>
-      <c r="C17" s="126"/>
-      <c r="D17" s="121" t="s">
+      <c r="A17" s="130"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="130"/>
+      <c r="D17" s="125" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="122" t="s">
+      <c r="E17" s="126" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="124" t="s">
+      <c r="F17" s="128" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="114"/>
-      <c r="H17" s="120"/>
-      <c r="I17" s="114"/>
-      <c r="J17" s="119" t="s">
+      <c r="G17" s="118"/>
+      <c r="H17" s="124"/>
+      <c r="I17" s="118"/>
+      <c r="J17" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="123" t="s">
+      <c r="K17" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="L17" s="124" t="s">
+      <c r="L17" s="128" t="s">
         <v>18</v>
       </c>
       <c r="M17" s="2"/>
@@ -7702,12 +7715,12 @@
       <c r="AU17" s="2"/>
     </row>
     <row r="18" spans="1:47" ht="12.75">
-      <c r="A18" s="120"/>
-      <c r="B18" s="120"/>
-      <c r="C18" s="120"/>
-      <c r="D18" s="120"/>
-      <c r="E18" s="120"/>
-      <c r="F18" s="114"/>
+      <c r="A18" s="124"/>
+      <c r="B18" s="124"/>
+      <c r="C18" s="124"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="118"/>
       <c r="G18" s="11">
         <v>5020301000</v>
       </c>
@@ -7717,9 +7730,9 @@
       <c r="I18" s="11">
         <v>5021202000</v>
       </c>
-      <c r="J18" s="120"/>
-      <c r="K18" s="120"/>
-      <c r="L18" s="114"/>
+      <c r="J18" s="124"/>
+      <c r="K18" s="124"/>
+      <c r="L18" s="118"/>
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
@@ -10918,14 +10931,14 @@
       <c r="D77" s="89"/>
       <c r="E77" s="89"/>
       <c r="F77" s="90"/>
-      <c r="G77" s="135" t="s">
+      <c r="G77" s="138" t="s">
         <v>101</v>
       </c>
-      <c r="H77" s="116"/>
-      <c r="I77" s="116"/>
-      <c r="J77" s="116"/>
-      <c r="K77" s="116"/>
-      <c r="L77" s="117"/>
+      <c r="H77" s="120"/>
+      <c r="I77" s="120"/>
+      <c r="J77" s="120"/>
+      <c r="K77" s="120"/>
+      <c r="L77" s="121"/>
       <c r="M77" s="2"/>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
@@ -11013,18 +11026,18 @@
     </row>
     <row r="79" spans="1:47" ht="14.25">
       <c r="A79" s="94"/>
-      <c r="B79" s="127" t="s">
+      <c r="B79" s="140" t="s">
         <v>102</v>
       </c>
-      <c r="C79" s="107"/>
+      <c r="C79" s="111"/>
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
       <c r="F79" s="92"/>
       <c r="G79" s="9"/>
-      <c r="H79" s="136" t="s">
+      <c r="H79" s="139" t="s">
         <v>103</v>
       </c>
-      <c r="I79" s="107"/>
+      <c r="I79" s="111"/>
       <c r="J79" s="9"/>
       <c r="K79" s="9"/>
       <c r="L79" s="93"/>
@@ -11124,10 +11137,10 @@
       <c r="F81" s="92"/>
       <c r="G81" s="9"/>
       <c r="H81" s="98"/>
-      <c r="I81" s="132" t="s">
+      <c r="I81" s="135" t="s">
         <v>105</v>
       </c>
-      <c r="J81" s="107"/>
+      <c r="J81" s="111"/>
       <c r="K81" s="9"/>
       <c r="L81" s="93"/>
       <c r="M81" s="2"/>
@@ -11177,10 +11190,10 @@
       <c r="F82" s="92"/>
       <c r="G82" s="9"/>
       <c r="H82" s="9"/>
-      <c r="I82" s="133" t="s">
+      <c r="I82" s="136" t="s">
         <v>107</v>
       </c>
-      <c r="J82" s="107"/>
+      <c r="J82" s="111"/>
       <c r="K82" s="9"/>
       <c r="L82" s="93"/>
       <c r="M82" s="2"/>
@@ -11271,18 +11284,18 @@
     <row r="84" spans="1:47" ht="14.25">
       <c r="A84" s="88"/>
       <c r="B84" s="89"/>
-      <c r="C84" s="134" t="s">
+      <c r="C84" s="137" t="s">
         <v>108</v>
       </c>
-      <c r="D84" s="113"/>
-      <c r="E84" s="113"/>
+      <c r="D84" s="117"/>
+      <c r="E84" s="117"/>
       <c r="F84" s="90"/>
       <c r="G84" s="89"/>
       <c r="H84" s="89"/>
-      <c r="I84" s="134" t="s">
+      <c r="I84" s="137" t="s">
         <v>109</v>
       </c>
-      <c r="J84" s="113"/>
+      <c r="J84" s="117"/>
       <c r="K84" s="89"/>
       <c r="L84" s="100"/>
       <c r="M84" s="2"/>

</xml_diff>